<commit_message>
fixed bug with writing daName to spreadsheet, and refactored the code
</commit_message>
<xml_diff>
--- a/newWorkbook.xlsx
+++ b/newWorkbook.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Device</t>
   </si>
@@ -22,13 +22,19 @@
     <t>127.0.0.1</t>
   </si>
   <si>
-    <t></t>
+    <t>vendor</t>
   </si>
   <si>
     <t>MZ Automation</t>
   </si>
   <si>
+    <t>swRev</t>
+  </si>
+  <si>
     <t>1.3.0</t>
+  </si>
+  <si>
+    <t>d</t>
   </si>
   <si>
     <t>libiec61850 server example</t>
@@ -363,13 +369,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
@@ -379,21 +394,10 @@
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="B6" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D6" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>